<commit_message>
feat(sheets): 민요 86곡 재판독 tsv·검수 xlsx·index 반영
- _작업/tsv: 86장 전부 판독(신규 7곡 + '하' 13곡 재판독)
- 검수 xlsx 86곡, sheets-index.json 갱신
- build_all.py(macOS용), 도구/check_tsv.py 추가, 진행이력 갱신
</commit_message>
<xml_diff>
--- a/sheets/민요/검수/궁초댕기.xlsx
+++ b/sheets/민요/검수/궁초댕기.xlsx
@@ -255,11 +255,7 @@
           <t xml:space="preserve">쪽</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">196</t>
-        </is>
-      </c>
+      <c r="B5" s="4"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -3908,10 +3904,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s=""/>
-      <c r="B1" s="">
-        <v>0</v>
-      </c>
+      <c r="A1" s="0"/>
     </row>
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="0"/>

</xml_diff>